<commit_message>
fix(7.2): ticket 15's reviews, and the empty Formula workbook
Fixes D294 and D295. The export's docstring names the workbook it copies
byte for byte, and it is "the empty Formula workbook", not a template,
which the glossary keeps for a user's script.

The offline policy now also finds a single-quoted external target, part
names in any case, a formula that fetches or links out, and a URL a
person typed in a cell. The hook reads text edits only, as before. The
steps follow the beginner reader's report.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/copilot/formula_workbook.xlsx
+++ b/copilot/formula_workbook.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Copilot turns this workbook into Hive, and the Hive into Toolbox code, without anyone explaining what the workbook is for. Make a copy of this file for each piece of work.</t>
+          <t>Copilot reads this workbook and writes Hive, the SQL your team's database runs, without anyone explaining what the workbook is for. Make a copy of this file for each piece of work.</t>
         </is>
       </c>
     </row>
@@ -484,63 +484,63 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1. On a sheet of its own, paste a sample of the raw data as values only (Home &gt; Paste &gt; Paste Values): one header row, one row per record, no blank rows, no merged cells.</t>
+          <t>1. For each table of raw data the work starts from, paste a sample on a sheet of its own, as values only (Home &gt; Paste &gt; Paste Values): one header row, one row per record, no blank rows, no merged cells. Paste only the columns that hold data, not the ones that hold formulas: you rebuild those in step 4.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2. Click inside it, press Ctrl+T and tick "My table has headers". Its name, under Table Design &gt; Table Name, can be whatever you like: Copilot keeps the names you give, and marks any it can't match to a Hive table for you to fill in.</t>
+          <t>2. Click inside it, press Ctrl+T and tick "My table has headers". If the data was already in a Table, keep that Table's name; if you know the database table it comes from, use that name. Otherwise any name will do, with no spaces (Table Design &gt; Table Name; on older Excel, Design under Table Tools). Copilot keeps the names you give, and marks any it can't match to a database table for you to fill in.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>3. Do steps 1 and 2 for every table of raw data before going on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Your calculations:</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>3. Add a column to the Table for each calculation, and write its formula once, in the first row, by column name, such as =[@units]*[@price]. Excel fills it down the column.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. A calculation that reads another Table, such as an XLOOKUP or a SUMIFS, is written the same way, naming the other Table: =XLOOKUP([@product_id], products[product_id], products[name]).</t>
+          <t>4. Add a column to a Table for each calculation, and write its formula once, in the first row. Click a cell in the same row rather than typing its address, and Excel writes it by column name, such as =[@units]*[@price]. Excel fills the formula down the column.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5. A Power Query step can do a calculation instead of a formula: Data &gt; From Table/Range, then Close &amp; Load. Copilot reads its steps too.</t>
+          <t>5. A calculation that reads another Table, such as an XLOOKUP or a SUMIFS, is written the same way, naming the other Table: =XLOOKUP([@product_id], products[product_id], products[name]). A summary of totals, such as a block of SUMIFS cells or a PivotTable, is rebuilt as a Table of its own: a column for what it groups by, one row per group, and a SUMIFS column for each figure.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6. Move each fixed value a formula uses, such as a rate typed in $B$3, into the Parameters Table, one row a value, and read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]).</t>
+          <t>6. Move each fixed value a formula uses into the Parameters Table, one row a value, whether it was typed in a cell such as $B$3 or inside a formula such as *0.2, and read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Values typed over a formula:</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>7. Power Query, if you use it, can do a calculation instead of a formula: Data &gt; From Table/Range, make the changes in the Power Query Editor, then Close &amp; Load to a new Table. Copilot reads its steps, and the new Table converts like any other. Skip this step if you don't use Power Query.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>7. A value typed over a formula in one row is converted as it is, for that row. Copilot needs to know which column or columns tell that Table's rows apart: add a row to the Keys Table, with the Table's name and those columns, separated by commas. A Table with no value typed over a formula needs no row in Keys.</t>
+          <t>8. A formula that reads the row above, such as a running total, or a cell outside a Table, can't be read as SQL: Copilot names it and leaves its column empty for you to finish.</t>
         </is>
       </c>
     </row>
@@ -554,21 +554,28 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>8. Take out anything you don't want converted: a Table, a column, a value typed over a formula. Whatever is left in a Table converts.</t>
+          <t>9. Take out anything you don't want converted: a Table, a column, a value typed over a formula. Whatever is left in a Table converts.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>9. Charts, PivotTables and anything outside a Table are left alone, and Copilot names them. Titles and notes can stay.</t>
+          <t>10. A value someone typed over a formula in one row is converted as it is, for that row. Find each in the original workbook (Ctrl+` shows formulas, so a typed value stands out) and type it over the formula in the same row here. Then add a row to the Keys Table: the Table's name, and the column or columns that tell its rows apart, separated by commas, such as job_runs | run_id, or sales | region, month. A Table with no value typed over a formula needs no row in Keys.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>10. Save the workbook, attach it in a Copilot chat with file 11 loaded, and ask Copilot to convert it.</t>
+          <t>11. Charts and anything outside a Table are left alone, and Copilot names them. Titles and notes can stay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>12. Save the workbook, attach it in a Copilot chat with Copilot file 11 loaded (with files 03, 04 and 05), and ask Copilot to convert it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sqlglot Composer 7.2, exported 2026-10-29 11:20
Generated from dev 0f52df08624e6a20f622190176027461c995e6f8 by tools/export_clean.py. Never edit this branch by hand.
</commit_message>
<xml_diff>
--- a/copilot/formula_workbook.xlsx
+++ b/copilot/formula_workbook.xlsx
@@ -540,7 +540,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>8. A formula that reads the row above, such as a running total, or a cell outside a Table, can't be read as SQL: Copilot names it and leaves its column empty for you to finish.</t>
+          <t>8. A formula that reads the row above, or a cell outside a Table, can't be read as SQL: Copilot names it and leaves its column empty for you to finish. Write a running total as =SUMIFS(t[v], t[d], "&lt;="&amp;[@d]), which Copilot can read.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>12. Save the workbook, attach it in a Copilot chat with Copilot file 11 loaded (with files 03, 04 and 05), and ask Copilot to convert it.</t>
+          <t>12. Save the workbook, attach it in a Copilot chat with Copilot files 11 and 12 loaded (with files 03, 04 and 05), and ask Copilot to convert it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(7.2): the empty Formula workbook says what Parameters and Keys are for
The user: "There are no instructions inside the xlsx template on what
Parameters and Keys are". The Steps sheet named them only in passing, at
steps 6 and 10, and their own sheets said nothing. The Steps sheet now opens
with a short section on both, and each sheet has a note beside its Table, in
column D so a row added to the Table never reaches it: what the Table is
for, an example, and when to leave it empty.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/copilot/formula_workbook.xlsx
+++ b/copilot/formula_workbook.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -477,103 +477,117 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Your data:</t>
+          <t>The Parameters and Keys sheets:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1. For each table of raw data the work starts from, paste a sample on a sheet of its own, as values only (Home &gt; Paste &gt; Paste Values): one header row, one row per record, no blank rows, no merged cells. Paste only the columns that hold data, not the ones that hold formulas: you rebuild those in step 4.</t>
+          <t>Parameters holds the fixed values your formulas use, such as a tax rate: one row each, its name under name and its value under value (step 6). Keys is only for a Table where a value was typed over a formula: it names the columns that tell that Table's rows apart, so Copilot can find the row (step 10). Both start empty, and stay empty if you need neither.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2. Click inside it, press Ctrl+T and tick "My table has headers". If the data was already in a Table, keep that Table's name; if you know the database table it comes from, use that name. Otherwise any name will do, with no spaces (Table Design &gt; Table Name; on older Excel, Design under Table Tools). Copilot keeps the names you give, and marks any it can't match to a database table for you to fill in.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Your data:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Do steps 1 and 2 for every table of raw data before going on.</t>
+          <t>1. For each table of raw data the work starts from, paste a sample on a sheet of its own, as values only (Home &gt; Paste &gt; Paste Values): one header row, one row per record, no blank rows, no merged cells. Paste only the columns that hold data, not the ones that hold formulas: you rebuild those in step 4.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Your calculations:</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2. Click inside it, press Ctrl+T and tick "My table has headers". If the data was already in a Table, keep that Table's name; if you know the database table it comes from, use that name. Otherwise any name will do, with no spaces (Table Design &gt; Table Name; on older Excel, Design under Table Tools). Copilot keeps the names you give, and marks any it can't match to a database table for you to fill in.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Add a column to a Table for each calculation, and write its formula once, in the first row. Click a cell in the same row rather than typing its address, and Excel writes it by column name, such as =[@units]*[@price]. Excel fills the formula down the column.</t>
+          <t>3. Do steps 1 and 2 for every table of raw data before going on.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>5. A calculation that reads another Table, such as an XLOOKUP or a SUMIFS, is written the same way, naming the other Table: =XLOOKUP([@product_id], products[product_id], products[name]). A summary of totals, such as a block of SUMIFS cells or a PivotTable, is rebuilt as a Table of its own: a column for what it groups by, one row per group, and a SUMIFS column for each figure.</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Your calculations:</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6. Move each fixed value a formula uses into the Parameters Table, one row a value, whether it was typed in a cell such as $B$3 or inside a formula such as *0.2, and read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]).</t>
+          <t>4. Add a column to a Table for each calculation, and write its formula once, in the first row. Click a cell in the same row rather than typing its address, and Excel writes it by column name, such as =[@units]*[@price]. Excel fills the formula down the column.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>7. Power Query, if you use it, can do a calculation instead of a formula: Data &gt; From Table/Range, make the changes in the Power Query Editor, then Close &amp; Load to a new Table. Copilot reads its steps, and the new Table converts like any other. Skip this step if you don't use Power Query.</t>
+          <t>5. A calculation that reads another Table, such as an XLOOKUP or a SUMIFS, is written the same way, naming the other Table: =XLOOKUP([@product_id], products[product_id], products[name]). A summary of totals, such as a block of SUMIFS cells or a PivotTable, is rebuilt as a Table of its own: a column for what it groups by, one row per group, and a SUMIFS column for each figure.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>8. A formula that reads the row above, or a cell outside a Table, can't be read as SQL: Copilot names it and leaves its column empty for you to finish. Write a running total as =SUMIFS(t[v], t[d], "&lt;="&amp;[@d]), which Copilot can read.</t>
+          <t>6. Move each fixed value a formula uses into the Parameters Table, one row a value, whether it was typed in a cell such as $B$3 or inside a formula such as *0.2, and read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Before you hand it over:</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>7. Power Query, if you use it, can do a calculation instead of a formula: Data &gt; From Table/Range, make the changes in the Power Query Editor, then Close &amp; Load to a new Table. Copilot reads its steps, and the new Table converts like any other. Skip this step if you don't use Power Query.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>9. Take out anything you don't want converted: a Table, a column, a value typed over a formula. Whatever is left in a Table converts.</t>
+          <t>8. A formula that reads the row above, or a cell outside a Table, can't be read as SQL: Copilot names it and leaves its column empty for you to finish. Write a running total as =SUMIFS(t[v], t[d], "&lt;="&amp;[@d]), which Copilot can read.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>10. A value someone typed over a formula in one row is converted as it is, for that row. Find each in the original workbook (Ctrl+` shows formulas, so a typed value stands out) and type it over the formula in the same row here. Then add a row to the Keys Table: the Table's name under table, and under key_columns the column or columns that tell its rows apart, separated by commas: job_runs and run_id, or sales and region, month. A Table with no value typed over a formula needs no row in Keys.</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Before you hand it over:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>11. Charts and anything outside a Table are left alone, and Copilot names them. Titles and notes can stay.</t>
+          <t>9. Take out anything you don't want converted: a Table, a column, a value typed over a formula. Whatever is left in a Table converts.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>10. A value someone typed over a formula in one row is converted as it is, for that row. Find each in the original workbook (Ctrl+` shows formulas, so a typed value stands out) and type it over the formula in the same row here. Then add a row to the Keys Table: the Table's name under table, and under key_columns the column or columns that tell its rows apart, separated by commas: job_runs and run_id, or sales and region, month. A Table with no value typed over a formula needs no row in Keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>11. Charts and anything outside a Table are left alone, and Copilot names them. Titles and notes can stay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>12. Save the workbook, attach it in a Copilot chat with Copilot files 11 and 12 loaded (with files 03, 04 and 05), and ask Copilot to convert it.</t>
         </is>
@@ -590,11 +604,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -606,6 +621,11 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Parameters: the fixed values your formulas use, one row each. Put its name under name and the value under value, such as tax_rate and 0.2, then read it by name in a formula: XLOOKUP("tax_rate", Parameters[name], Parameters[value]). Leave the Table empty if no formula uses a fixed value. See step 6 on the Steps sheet.</t>
         </is>
       </c>
     </row>
@@ -623,11 +643,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -639,6 +660,11 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>key_columns</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Keys: only for a Table where a value was typed over a formula in one row. Add a row: that Table's name under table, and under key_columns the column or columns that tell its rows apart, separated by commas, such as job_runs and run_id. Copilot uses them to find the row. A Table with no value typed over a formula needs no row here. See step 10 on the Steps sheet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(7.2): the workbook says how to fill Parameters and Keys, from the beginner reader
One Keys row per Table, however many values were typed over in it; the two
examples set apart; only typed columns as keys, and a Table with no column
telling its rows apart left out of Keys, as Copilot then matches on every
typed column; the sample must hold the typed-over row; Parameters one row per
value, the formula changed to read it, and 0.2 rather than 20%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/copilot/formula_workbook.xlsx
+++ b/copilot/formula_workbook.xlsx
@@ -484,7 +484,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Parameters holds the fixed values your formulas use, such as a tax rate: one row each, its name under name and its value under value (step 6). Keys is only for a Table where a value was typed over a formula: it names the columns that tell that Table's rows apart, so Copilot can find the row (step 10). Both start empty, and stay empty if you need neither.</t>
+          <t>Parameters holds the fixed values your formulas use, such as a tax rate: one row each, its name under name and its value under value (step 6). Keys is only for a Table where a value was typed over a formula: it names the columns that tell that Table's rows apart, so Copilot can find the row the typed value belongs to (step 10). Both start empty, and stay empty if you need neither.</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>6. Move each fixed value a formula uses into the Parameters Table, one row a value, whether it was typed in a cell such as $B$3 or inside a formula such as *0.2, and read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]).</t>
+          <t>6. Move each fixed value a formula uses into the Parameters Table, one row per value, whether it was typed in a cell such as $B$3 or inside a formula such as *0.2, and change the formula to read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]). Write a value as a plain number or text: 0.2, not 20%.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>10. A value someone typed over a formula in one row is converted as it is, for that row. Find each in the original workbook (Ctrl+` shows formulas, so a typed value stands out) and type it over the formula in the same row here. Then add a row to the Keys Table: the Table's name under table, and under key_columns the column or columns that tell its rows apart, separated by commas: job_runs and run_id, or sales and region, month. A Table with no value typed over a formula needs no row in Keys.</t>
+          <t>10. A value someone typed over a formula in one row is converted as it is, for that row. Find each in the original workbook (Ctrl+` shows formulas, so a typed value stands out) and type it over the formula in the same row here, making sure your sample holds that row. Then add one row to the Keys Table for that Table, however many values were typed over in it: the Table's name under table, and under key_columns the typed column or columns that tell its rows apart, separated by commas. For example, job_runs with run_id; or sales with region, month. If no column tells the rows apart, leave the Table out of Keys: Copilot then matches the row on all its typed columns. A Table with no value typed over a formula needs no row in Keys.</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Parameters: the fixed values your formulas use, one row each. Put its name under name and the value under value, such as tax_rate and 0.2, then read it by name in a formula: XLOOKUP("tax_rate", Parameters[name], Parameters[value]). Leave the Table empty if no formula uses a fixed value. See step 6 on the Steps sheet.</t>
+          <t>Parameters: the fixed values your formulas use, one row per value. Put its name under name and the value under value, such as tax_rate and 0.2 (a plain number, not 20%), then read it by name in a formula: XLOOKUP("tax_rate", Parameters[name], Parameters[value]). Leave the Table empty if no formula uses a fixed value. See step 6 on the Steps sheet.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Keys: only for a Table where a value was typed over a formula in one row. Add a row: that Table's name under table, and under key_columns the column or columns that tell its rows apart, separated by commas, such as job_runs and run_id. Copilot uses them to find the row. A Table with no value typed over a formula needs no row here. See step 10 on the Steps sheet.</t>
+          <t>Keys: only for a Table where a value was typed over a formula. Add one row for that Table, however many values were typed over in it: the Table's name under table, and under key_columns the typed column or columns that tell its rows apart, separated by commas, such as job_runs with run_id, or sales with region, month. Copilot uses them to find the row a typed value belongs to. If no column tells the rows apart, leave the Table out. A Table with no value typed over a formula needs no row here. See step 10 on the Steps sheet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sqlglot Composer 7.2, exported 2026-10-29 14:21
Generated from dev 10cfdc622bd61d04d64042cd123a66a8a87894c1 by tools/export_clean.py. Never edit this branch by hand.
</commit_message>
<xml_diff>
--- a/copilot/formula_workbook.xlsx
+++ b/copilot/formula_workbook.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -477,103 +477,117 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Your data:</t>
+          <t>The Parameters and Keys sheets:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1. For each table of raw data the work starts from, paste a sample on a sheet of its own, as values only (Home &gt; Paste &gt; Paste Values): one header row, one row per record, no blank rows, no merged cells. Paste only the columns that hold data, not the ones that hold formulas: you rebuild those in step 4.</t>
+          <t>Parameters holds the fixed values your formulas use, such as a tax rate: one row each, its name under name and its value under value (step 6). Keys is only for a Table where a value was typed over a formula: it names the columns that tell that Table's rows apart, so Copilot can find the row the typed value belongs to (step 10). Both start empty, and stay empty if you need neither.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2. Click inside it, press Ctrl+T and tick "My table has headers". If the data was already in a Table, keep that Table's name; if you know the database table it comes from, use that name. Otherwise any name will do, with no spaces (Table Design &gt; Table Name; on older Excel, Design under Table Tools). Copilot keeps the names you give, and marks any it can't match to a database table for you to fill in.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Your data:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Do steps 1 and 2 for every table of raw data before going on.</t>
+          <t>1. For each table of raw data the work starts from, paste a sample on a sheet of its own, as values only (Home &gt; Paste &gt; Paste Values): one header row, one row per record, no blank rows, no merged cells. Paste only the columns that hold data, not the ones that hold formulas: you rebuild those in step 4.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Your calculations:</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2. Click inside it, press Ctrl+T and tick "My table has headers". If the data was already in a Table, keep that Table's name; if you know the database table it comes from, use that name. Otherwise any name will do, with no spaces (Table Design &gt; Table Name; on older Excel, Design under Table Tools). Copilot keeps the names you give, and marks any it can't match to a database table for you to fill in.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Add a column to a Table for each calculation, and write its formula once, in the first row. Click a cell in the same row rather than typing its address, and Excel writes it by column name, such as =[@units]*[@price]. Excel fills the formula down the column.</t>
+          <t>3. Do steps 1 and 2 for every table of raw data before going on.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>5. A calculation that reads another Table, such as an XLOOKUP or a SUMIFS, is written the same way, naming the other Table: =XLOOKUP([@product_id], products[product_id], products[name]). A summary of totals, such as a block of SUMIFS cells or a PivotTable, is rebuilt as a Table of its own: a column for what it groups by, one row per group, and a SUMIFS column for each figure.</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Your calculations:</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6. Move each fixed value a formula uses into the Parameters Table, one row a value, whether it was typed in a cell such as $B$3 or inside a formula such as *0.2, and read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]).</t>
+          <t>4. Add a column to a Table for each calculation, and write its formula once, in the first row. Click a cell in the same row rather than typing its address, and Excel writes it by column name, such as =[@units]*[@price]. Excel fills the formula down the column.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>7. Power Query, if you use it, can do a calculation instead of a formula: Data &gt; From Table/Range, make the changes in the Power Query Editor, then Close &amp; Load to a new Table. Copilot reads its steps, and the new Table converts like any other. Skip this step if you don't use Power Query.</t>
+          <t>5. A calculation that reads another Table, such as an XLOOKUP or a SUMIFS, is written the same way, naming the other Table: =XLOOKUP([@product_id], products[product_id], products[name]). A summary of totals, such as a block of SUMIFS cells or a PivotTable, is rebuilt as a Table of its own: a column for what it groups by, one row per group, and a SUMIFS column for each figure.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>8. A formula that reads the row above, or a cell outside a Table, can't be read as SQL: Copilot names it and leaves its column empty for you to finish. Write a running total as =SUMIFS(t[v], t[d], "&lt;="&amp;[@d]), which Copilot can read.</t>
+          <t>6. Move each fixed value a formula uses into the Parameters Table, one row per value, whether it was typed in a cell such as $B$3 or inside a formula such as *0.2, and change the formula to read it by name: =XLOOKUP("tax_rate", Parameters[name], Parameters[value]). Write a value as a plain number or text: 0.2, not 20%.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Before you hand it over:</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>7. Power Query, if you use it, can do a calculation instead of a formula: Data &gt; From Table/Range, make the changes in the Power Query Editor, then Close &amp; Load to a new Table. Copilot reads its steps, and the new Table converts like any other. Skip this step if you don't use Power Query.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>9. Take out anything you don't want converted: a Table, a column, a value typed over a formula. Whatever is left in a Table converts.</t>
+          <t>8. A formula that reads the row above, or a cell outside a Table, can't be read as SQL: Copilot names it and leaves its column empty for you to finish. Write a running total as =SUMIFS(t[v], t[d], "&lt;="&amp;[@d]), which Copilot can read.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>10. A value someone typed over a formula in one row is converted as it is, for that row. Find each in the original workbook (Ctrl+` shows formulas, so a typed value stands out) and type it over the formula in the same row here. Then add a row to the Keys Table: the Table's name under table, and under key_columns the column or columns that tell its rows apart, separated by commas: job_runs and run_id, or sales and region, month. A Table with no value typed over a formula needs no row in Keys.</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Before you hand it over:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>11. Charts and anything outside a Table are left alone, and Copilot names them. Titles and notes can stay.</t>
+          <t>9. Take out anything you don't want converted: a Table, a column, a value typed over a formula. Whatever is left in a Table converts.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>10. A value someone typed over a formula in one row is converted as it is, for that row. Find each in the original workbook (Ctrl+` shows formulas, so a typed value stands out) and type it over the formula in the same row here, making sure your sample holds that row. Then add one row to the Keys Table for that Table, however many values were typed over in it: the Table's name under table, and under key_columns the typed column or columns that tell its rows apart, separated by commas. For example, job_runs with run_id; or sales with region, month. If no column tells the rows apart, leave the Table out of Keys: Copilot then matches the row on all its typed columns. A Table with no value typed over a formula needs no row in Keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>11. Charts and anything outside a Table are left alone, and Copilot names them. Titles and notes can stay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>12. Save the workbook, attach it in a Copilot chat with Copilot files 11 and 12 loaded (with files 03, 04 and 05), and ask Copilot to convert it.</t>
         </is>
@@ -590,11 +604,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -606,6 +621,11 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Parameters: the fixed values your formulas use, one row per value. Put its name under name and the value under value, such as tax_rate and 0.2 (a plain number, not 20%), then read it by name in a formula: XLOOKUP("tax_rate", Parameters[name], Parameters[value]). Leave the Table empty if no formula uses a fixed value. See step 6 on the Steps sheet.</t>
         </is>
       </c>
     </row>
@@ -623,11 +643,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -639,6 +660,11 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>key_columns</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Keys: only for a Table where a value was typed over a formula. Add one row for that Table, however many values were typed over in it: the Table's name under table, and under key_columns the typed column or columns that tell its rows apart, separated by commas, such as job_runs with run_id, or sales with region, month. Copilot uses them to find the row a typed value belongs to. If no column tells the rows apart, leave the Table out. A Table with no value typed over a formula needs no row here. See step 10 on the Steps sheet.</t>
         </is>
       </c>
     </row>

</xml_diff>